<commit_message>
Mise à jour des bases coûts et nouvelle version tous
</commit_message>
<xml_diff>
--- a/Remote/ug16/Commun/dist_users.xlsx
+++ b/Remote/ug16/Commun/dist_users.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Mickaël\Documents\GitHub\ductaironline\Remote\ug16\Commun\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8E5A858-79C1-44B9-8704-F5758A4619C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92556E9D-79EF-432B-81F0-84E69490FBCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FB319E84-7C88-461F-9183-805C577E13FE}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="94">
   <si>
     <t>ID</t>
   </si>
@@ -871,7 +871,7 @@
         <v>31</v>
       </c>
       <c r="U2" t="s">
-        <v>32</v>
+        <v>92</v>
       </c>
       <c r="V2" s="3" t="s">
         <v>93</v>
@@ -941,7 +941,6 @@
       <c r="U3" t="s">
         <v>32</v>
       </c>
-      <c r="V3" s="3"/>
     </row>
     <row r="4" spans="1:22">
       <c r="A4">
@@ -1005,7 +1004,10 @@
         <v>81</v>
       </c>
       <c r="U4" t="s">
-        <v>32</v>
+        <v>92</v>
+      </c>
+      <c r="V4" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:22" ht="14.25">
@@ -1070,9 +1072,11 @@
         <v>61645</v>
       </c>
       <c r="U5" t="s">
-        <v>32</v>
-      </c>
-      <c r="V5" s="3"/>
+        <v>92</v>
+      </c>
+      <c r="V5" s="3" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="6" spans="1:22">
       <c r="A6">
@@ -1136,7 +1140,10 @@
         <v>88</v>
       </c>
       <c r="U6" t="s">
-        <v>32</v>
+        <v>92</v>
+      </c>
+      <c r="V6" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:22" ht="14.25">
@@ -1335,7 +1342,7 @@
         <v>59</v>
       </c>
       <c r="U9" t="s">
-        <v>32</v>
+        <v>92</v>
       </c>
       <c r="V9" s="3" t="s">
         <v>93</v>
@@ -1419,6 +1426,7 @@
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="Q5" r:id="rId1" xr:uid="{3463426B-B927-4144-874B-D4A6866CFF40}"/>
+    <hyperlink ref="V7" r:id="rId2" xr:uid="{A62A8E25-0288-4E95-A80A-240FB587558B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>